<commit_message>
2024-12-03-feat: add half analysis
</commit_message>
<xml_diff>
--- a/assets/desc.xlsx
+++ b/assets/desc.xlsx
@@ -425,71 +425,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>surface_type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>liquid_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>diameter</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>height</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fall_point_type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>area</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>circumstance</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>circularity</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>finger_num</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>velocity</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>circle_radius</t>
         </is>
@@ -540,6 +545,9 @@
       <c r="N2" t="n">
         <v>812</v>
       </c>
+      <c r="O2" t="n">
+        <v>812</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -548,42 +556,45 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>405.5</v>
+      </c>
+      <c r="C3" t="n">
         <v>3.056650246305419</v>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>19.89901477832512</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>32.19211822660098</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>5.269704433497537</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>120.8386699507389</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.02416773399014779</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>1.00472459408867e-05</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.01660210667943128</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.4721465972935146</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>17.58128078817734</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.2510837438423645</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.001781187192118227</v>
       </c>
     </row>
@@ -594,42 +605,45 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>234.5485024467221</v>
+      </c>
+      <c r="C4" t="n">
         <v>2.510003190361046</v>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
       <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
         <v>2.631432688172558</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>9.136452211303526</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>2.717240642014267</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>25.9838199148173</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.005196763982963459</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>3.498367557234918e-06</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.004213183586972885</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.1211834705628292</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>5.538747656994963</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>3.177056980267059</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.0003033004954879778</v>
       </c>
     </row>
@@ -646,36 +660,39 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>18</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>20</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>91</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.0182</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>2.184048e-06</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.0100176986231803</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.1450933693301122</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>3</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>-37.86</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>0.00084</v>
       </c>
     </row>
@@ -686,42 +703,45 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>202.75</v>
+      </c>
+      <c r="C6" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
       <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>18</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>20</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>4</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>106</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>0.0212</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>7.105968000000001e-06</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.01292718125259868</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.3796681850834678</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>14</v>
       </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
       <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
         <v>0.001524</v>
       </c>
     </row>
@@ -732,42 +752,45 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>405.5</v>
+      </c>
+      <c r="C7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
       <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>18</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>40</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>5</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>122</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>0.0244</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>1.0139004e-05</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>0.01624416433596605</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.4674645876033258</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>18</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>0.06</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.0018</v>
       </c>
     </row>
@@ -778,42 +801,45 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>608.25</v>
+      </c>
+      <c r="C8" t="n">
         <v>5</v>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
       <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>20</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>40</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>7</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>131</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>0.0262</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>1.3317066e-05</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>0.0200551759700775</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.5606603453412629</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>22</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>0.18</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.002076</v>
       </c>
     </row>
@@ -824,42 +850,45 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>811</v>
+      </c>
+      <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>25</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>40</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>9</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>364</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>0.0728</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>1.636704e-05</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>0.03061915467453</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.7702187513147767</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>33</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>9.84</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>0.00228</v>
       </c>
     </row>

</xml_diff>